<commit_message>
feat: add project links and PDF archiving
</commit_message>
<xml_diff>
--- a/02_源码和说明/2026-乙方宝招标信息统计.xlsx
+++ b/02_源码和说明/2026-乙方宝招标信息统计.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="公告详情" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="公告详情" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -157,7 +157,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -224,6 +224,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -770,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="30" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -784,69 +788,93 @@
     <col width="30" customWidth="1" style="5" min="9" max="9"/>
     <col width="55" customWidth="1" style="5" min="10" max="10"/>
     <col width="36" customWidth="1" style="1" min="11" max="11"/>
-    <col width="30" customWidth="1" style="1" min="12" max="12"/>
-    <col width="30" customWidth="1" style="1" min="13" max="16384"/>
+    <col width="22" customWidth="1" style="1" min="12" max="12"/>
+    <col width="12" customWidth="1" style="1" min="13" max="16384"/>
+    <col hidden="1" width="13" customWidth="1" style="5" min="14" max="14"/>
+    <col hidden="1" width="13" customWidth="1" style="5" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1" s="5">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>序号</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>日期</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>项目名称</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="24" t="inlineStr">
         <is>
           <t>建设单位</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="24" t="inlineStr">
         <is>
           <t>项目位置</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="24" t="inlineStr">
         <is>
           <t>资质</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="24" t="inlineStr">
         <is>
           <t>报名时间</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="H1" s="24" t="inlineStr">
         <is>
           <t>投标截止时间</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="I1" s="24" t="inlineStr">
         <is>
           <t>基本情况</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="24" t="inlineStr">
         <is>
           <t>相关性</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="K1" s="24" t="inlineStr">
         <is>
           <t>备注</t>
+        </is>
+      </c>
+      <c r="L1" s="24" t="inlineStr">
+        <is>
+          <t>项目编号</t>
+        </is>
+      </c>
+      <c r="M1" s="24" t="inlineStr">
+        <is>
+          <t>下载</t>
+        </is>
+      </c>
+      <c r="N1" s="0" t="inlineStr">
+        <is>
+          <t>详情网址</t>
+        </is>
+      </c>
+      <c r="O1" s="0" t="inlineStr">
+        <is>
+          <t>导出网址</t>
         </is>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="5">
-      <c r="A2" s="6" t="n"/>
+      <c r="A2" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="B2" s="6" t="n"/>
       <c r="C2" s="6" t="n"/>
       <c r="D2" s="6" t="n"/>
@@ -857,6 +885,8 @@
       <c r="I2" s="9" t="n"/>
       <c r="J2" s="9" t="n"/>
       <c r="K2" s="9" t="n"/>
+      <c r="L2" s="9" t="n"/>
+      <c r="M2" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -870,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="5" min="1" max="1"/>
@@ -878,6 +908,8 @@
     <col width="16" customWidth="1" style="5" min="3" max="3"/>
     <col width="120" customWidth="1" style="5" min="4" max="4"/>
     <col width="18" customWidth="1" style="5" min="5" max="5"/>
+    <col width="22" customWidth="1" style="5" min="6" max="6"/>
+    <col hidden="1" width="13" customWidth="1" style="5" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -904,6 +936,16 @@
       <c r="E1" s="21" t="inlineStr">
         <is>
           <t>返回主表</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>项目编号</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>链接键</t>
         </is>
       </c>
     </row>

</xml_diff>